<commit_message>
Phase 2: wire S01/S02/S03/S16/S33 Excel generators to the database
s01_assumptions, s02_equipment, s03_supplier, s16_risk, and
s33_portfolio_register now read their data via db.py's list_*/get_*
functions instead of hardcoded Python literals. Sheet layout and
formula logic are unchanged; only the data source moved. Also
includes the seed_from_current.py depreciation-method fix from
Phase 1 that hadn't been committed yet.

Full workbook rebuilt and re-validated: 36 sheets, 9203 formula
cells evaluated, 0 errors. Rollup values (PRG-001/PRG-002 CapEx,
budget, portfolio totals) match the database exactly, confirming
no numeric drift from the pre-migration workbook.
</commit_message>
<xml_diff>
--- a/downloads/CapEx_StrategicSC_Portfolio.xlsx
+++ b/downloads/CapEx_StrategicSC_Portfolio.xlsx
@@ -9245,7 +9245,7 @@
         </is>
       </c>
       <c r="B6" s="62">
-        <f>'S01_Disclaimer_Assumptions'!$B$30</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$29</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -9261,7 +9261,7 @@
         </is>
       </c>
       <c r="B7" s="62">
-        <f>'S01_Disclaimer_Assumptions'!$B$31</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$30</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -9293,7 +9293,7 @@
         </is>
       </c>
       <c r="B9" s="62">
-        <f>'S01_Disclaimer_Assumptions'!$B$32</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$31</f>
         <v/>
       </c>
       <c r="D9" t="inlineStr">
@@ -14872,15 +14872,15 @@
         </is>
       </c>
       <c r="B6" s="93">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="C6" s="93">
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
+        <v/>
+      </c>
+      <c r="D6" s="93">
         <f>'S01_Disclaimer_Assumptions'!$B$58</f>
-        <v/>
-      </c>
-      <c r="D6" s="93">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
         <v/>
       </c>
       <c r="E6" t="inlineStr">
@@ -14896,15 +14896,15 @@
         </is>
       </c>
       <c r="B7" s="93">
-        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
         <v/>
       </c>
       <c r="C7" s="93">
+        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <v/>
+      </c>
+      <c r="D7" s="93">
         <f>'S01_Disclaimer_Assumptions'!$B$60</f>
-        <v/>
-      </c>
-      <c r="D7" s="93">
-        <f>'S01_Disclaimer_Assumptions'!$B$61</f>
         <v/>
       </c>
       <c r="E7" t="inlineStr">
@@ -15009,11 +15009,11 @@
         </is>
       </c>
       <c r="D11" s="94">
-        <f>'S02_Equipment_Portfolio'!I5/'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S02_Equipment_Portfolio'!I5/'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="E11" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="F11" s="31">
@@ -15021,7 +15021,7 @@
         <v/>
       </c>
       <c r="G11" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
         <v/>
       </c>
       <c r="H11" s="31">
@@ -15033,7 +15033,7 @@
         <v/>
       </c>
       <c r="J11" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
         <v/>
       </c>
       <c r="K11" s="31">
@@ -15071,11 +15071,11 @@
         </is>
       </c>
       <c r="D12" s="94">
-        <f>'S02_Equipment_Portfolio'!I6/'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S02_Equipment_Portfolio'!I6/'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="E12" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="F12" s="31">
@@ -15083,7 +15083,7 @@
         <v/>
       </c>
       <c r="G12" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
         <v/>
       </c>
       <c r="H12" s="31">
@@ -15095,7 +15095,7 @@
         <v/>
       </c>
       <c r="J12" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
         <v/>
       </c>
       <c r="K12" s="31">
@@ -15133,11 +15133,11 @@
         </is>
       </c>
       <c r="D13" s="94">
-        <f>'S02_Equipment_Portfolio'!I8*'S01_Disclaimer_Assumptions'!$B$57</f>
+        <f>'S02_Equipment_Portfolio'!I8*'S01_Disclaimer_Assumptions'!$B$56</f>
         <v/>
       </c>
       <c r="E13" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
         <v/>
       </c>
       <c r="F13" s="31">
@@ -15145,7 +15145,7 @@
         <v/>
       </c>
       <c r="G13" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$60</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
         <v/>
       </c>
       <c r="H13" s="31">
@@ -15157,7 +15157,7 @@
         <v/>
       </c>
       <c r="J13" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$61</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$60</f>
         <v/>
       </c>
       <c r="K13" s="31">
@@ -15195,11 +15195,11 @@
         </is>
       </c>
       <c r="D14" s="94">
-        <f>'S02_Equipment_Portfolio'!I10*'S01_Disclaimer_Assumptions'!$B$57</f>
+        <f>'S02_Equipment_Portfolio'!I10*'S01_Disclaimer_Assumptions'!$B$56</f>
         <v/>
       </c>
       <c r="E14" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
         <v/>
       </c>
       <c r="F14" s="31">
@@ -15207,7 +15207,7 @@
         <v/>
       </c>
       <c r="G14" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$60</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
         <v/>
       </c>
       <c r="H14" s="31">
@@ -15219,7 +15219,7 @@
         <v/>
       </c>
       <c r="J14" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$61</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$60</f>
         <v/>
       </c>
       <c r="K14" s="31">
@@ -15257,11 +15257,11 @@
         </is>
       </c>
       <c r="D15" s="94">
-        <f>'S02_Equipment_Portfolio'!I11/'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S02_Equipment_Portfolio'!I11/'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="E15" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="F15" s="31">
@@ -15269,7 +15269,7 @@
         <v/>
       </c>
       <c r="G15" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
         <v/>
       </c>
       <c r="H15" s="31">
@@ -15281,7 +15281,7 @@
         <v/>
       </c>
       <c r="J15" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
         <v/>
       </c>
       <c r="K15" s="31">
@@ -15321,11 +15321,11 @@
         </is>
       </c>
       <c r="D16" s="94">
-        <f>'S02_Equipment_Portfolio'!I12/'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S02_Equipment_Portfolio'!I12/'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="E16" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="F16" s="31">
@@ -15333,7 +15333,7 @@
         <v/>
       </c>
       <c r="G16" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
         <v/>
       </c>
       <c r="H16" s="31">
@@ -15345,7 +15345,7 @@
         <v/>
       </c>
       <c r="J16" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
         <v/>
       </c>
       <c r="K16" s="31">
@@ -15383,11 +15383,11 @@
         </is>
       </c>
       <c r="D17" s="94">
-        <f>'S02_Equipment_Portfolio'!I13/'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S02_Equipment_Portfolio'!I13/'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="E17" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="F17" s="31">
@@ -15395,7 +15395,7 @@
         <v/>
       </c>
       <c r="G17" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
         <v/>
       </c>
       <c r="H17" s="31">
@@ -15407,7 +15407,7 @@
         <v/>
       </c>
       <c r="J17" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
         <v/>
       </c>
       <c r="K17" s="31">
@@ -15445,11 +15445,11 @@
         </is>
       </c>
       <c r="D18" s="94">
-        <f>'S02_Equipment_Portfolio'!I16*'S01_Disclaimer_Assumptions'!$B$57</f>
+        <f>'S02_Equipment_Portfolio'!I16*'S01_Disclaimer_Assumptions'!$B$56</f>
         <v/>
       </c>
       <c r="E18" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
         <v/>
       </c>
       <c r="F18" s="31">
@@ -15457,7 +15457,7 @@
         <v/>
       </c>
       <c r="G18" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$60</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
         <v/>
       </c>
       <c r="H18" s="31">
@@ -15469,7 +15469,7 @@
         <v/>
       </c>
       <c r="J18" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$61</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$60</f>
         <v/>
       </c>
       <c r="K18" s="31">
@@ -15507,11 +15507,11 @@
         </is>
       </c>
       <c r="D19" s="94">
-        <f>'S02_Equipment_Portfolio'!I17/'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S02_Equipment_Portfolio'!I17/'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="E19" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="F19" s="31">
@@ -15519,7 +15519,7 @@
         <v/>
       </c>
       <c r="G19" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
         <v/>
       </c>
       <c r="H19" s="31">
@@ -15531,7 +15531,7 @@
         <v/>
       </c>
       <c r="J19" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
         <v/>
       </c>
       <c r="K19" s="31">
@@ -15569,11 +15569,11 @@
         </is>
       </c>
       <c r="D20" s="94">
-        <f>'S02_Equipment_Portfolio'!I19/'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S02_Equipment_Portfolio'!I19/'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="E20" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$56</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$55</f>
         <v/>
       </c>
       <c r="F20" s="31">
@@ -15581,7 +15581,7 @@
         <v/>
       </c>
       <c r="G20" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$57</f>
         <v/>
       </c>
       <c r="H20" s="31">
@@ -15593,7 +15593,7 @@
         <v/>
       </c>
       <c r="J20" s="33">
-        <f>'S01_Disclaimer_Assumptions'!$B$59</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$58</f>
         <v/>
       </c>
       <c r="K20" s="31">
@@ -22738,7 +22738,7 @@
         <v/>
       </c>
       <c r="O6" s="31">
-        <f>N6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P6" s="8" t="inlineStr">
@@ -22804,7 +22804,7 @@
         <v/>
       </c>
       <c r="O7" s="31">
-        <f>N7*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N7*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P7" s="8" t="inlineStr">
@@ -22870,7 +22870,7 @@
         <v/>
       </c>
       <c r="O8" s="31">
-        <f>N8*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N8*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P8" s="8" t="inlineStr">
@@ -22936,7 +22936,7 @@
         <v/>
       </c>
       <c r="O9" s="31">
-        <f>N9*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N9*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P9" s="8" t="inlineStr">
@@ -23002,7 +23002,7 @@
         <v/>
       </c>
       <c r="O10" s="31">
-        <f>N10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P10" s="8" t="inlineStr">
@@ -23068,7 +23068,7 @@
         <v/>
       </c>
       <c r="O11" s="31">
-        <f>N11*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N11*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P11" s="8" t="inlineStr">
@@ -23134,7 +23134,7 @@
         <v/>
       </c>
       <c r="O12" s="31">
-        <f>N12*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N12*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P12" s="8" t="inlineStr">
@@ -23200,7 +23200,7 @@
         <v/>
       </c>
       <c r="O13" s="31">
-        <f>N13*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N13*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P13" s="8" t="inlineStr">
@@ -23266,7 +23266,7 @@
         <v/>
       </c>
       <c r="O14" s="31">
-        <f>N14*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N14*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P14" s="8" t="inlineStr">
@@ -23332,7 +23332,7 @@
         <v/>
       </c>
       <c r="O15" s="31">
-        <f>N15*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N15*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P15" s="8" t="inlineStr">
@@ -23398,7 +23398,7 @@
         <v/>
       </c>
       <c r="O16" s="31">
-        <f>N16*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N16*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P16" s="8" t="inlineStr">
@@ -23464,7 +23464,7 @@
         <v/>
       </c>
       <c r="O17" s="31">
-        <f>N17*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>N17*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="P17" s="8" t="inlineStr">
@@ -27371,7 +27371,7 @@
         <v/>
       </c>
       <c r="J6" s="31">
-        <f>H6+I6+42000+95000</f>
+        <f>H6+I6+42000.0+95000.0</f>
         <v/>
       </c>
       <c r="K6" s="47" t="n">
@@ -34938,7 +34938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -35262,13 +35262,11 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>CapEx Depreciation Method</t>
-        </is>
-      </c>
-      <c r="B18" s="43" t="inlineStr">
-        <is>
-          <t>MACRS 7-yr</t>
-        </is>
+          <t>Inflation Rate</t>
+        </is>
+      </c>
+      <c r="B18" s="47" t="n">
+        <v>0.025</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
@@ -35277,7 +35275,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Finance / Tax Counsel guidance</t>
+          <t>Corporate finance planning assumption</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -35287,87 +35285,87 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Per AR Summary financial justification</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Inflation Rate</t>
-        </is>
-      </c>
-      <c r="B19" s="47" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Corporate finance planning assumption</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
+          <t>Used to escalate Year 2-10 OpEx in TCO model</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>LABOR RATES</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Source / Basis</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Date Validated</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Fabrication Shop Rate</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="n">
+        <v>95</v>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>USD/hr</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Supplier benchmarking; 2024 MW industrial rate</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Used to escalate Year 2-10 OpEx in TCO model</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>LABOR RATES</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Source / Basis</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Date Validated</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Used in Should-Cost labor model (S04)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Fabrication Shop Rate</t>
+          <t>Engineering Labor Rate</t>
         </is>
       </c>
       <c r="B23" s="48" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
@@ -35376,7 +35374,7 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Supplier benchmarking; 2024 MW industrial rate</t>
+          <t>Internal engineering rate card Rev 2024</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -35386,18 +35384,18 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Used in Should-Cost labor model (S04)</t>
+          <t>Used in NRE and program labor estimates</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Engineering Labor Rate</t>
+          <t>Installation Labor Rate</t>
         </is>
       </c>
       <c r="B24" s="48" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
@@ -35406,7 +35404,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Internal engineering rate card Rev 2024</t>
+          <t>Facilities contractor rate card</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -35416,18 +35414,18 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Used in NRE and program labor estimates</t>
+          <t>Used in on-site installation cost estimates</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Installation Labor Rate</t>
+          <t>Field Service Rate (Supplier)</t>
         </is>
       </c>
       <c r="B25" s="48" t="n">
-        <v>85</v>
+        <v>175</v>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
@@ -35436,7 +35434,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Facilities contractor rate card</t>
+          <t>Supplier FSE rate benchmark</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -35446,87 +35444,87 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Used in on-site installation cost estimates</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Field Service Rate (Supplier)</t>
-        </is>
-      </c>
-      <c r="B26" s="48" t="n">
-        <v>175</v>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>USD/hr</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>Supplier FSE rate benchmark</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
+          <t>Used in downtime / MTTR cost modelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>EQUIPMENT PERFORMANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Source / Basis</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Date Validated</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Equipment Uptime Target</t>
+        </is>
+      </c>
+      <c r="B29" s="47" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Program engineering specification</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Used in downtime / MTTR cost modelling</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>EQUIPMENT PERFORMANCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Source / Basis</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Date Validated</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>92% uptime = 608 downtime hrs/yr basis for MTBF model</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Equipment Uptime Target</t>
+          <t>Planned Maintenance Downtime</t>
         </is>
       </c>
       <c r="B30" s="47" t="n">
-        <v>0.92</v>
+        <v>0.04</v>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
@@ -35535,7 +35533,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Program engineering specification</t>
+          <t>Maintenance planning schedule</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
@@ -35545,18 +35543,18 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>92% uptime = 608 downtime hrs/yr basis for MTBF model</t>
+          <t>4% of annual hours allocated to preventive maintenance</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Planned Maintenance Downtime</t>
+          <t>Process Yield Assumption</t>
         </is>
       </c>
       <c r="B31" s="47" t="n">
-        <v>0.04</v>
+        <v>0.96</v>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
@@ -35565,7 +35563,7 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Maintenance planning schedule</t>
+          <t>Engineering process spec</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
@@ -35575,117 +35573,117 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>4% of annual hours allocated to preventive maintenance</t>
+          <t>Used in capacity model to calculate effective throughput</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Process Yield Assumption</t>
-        </is>
-      </c>
-      <c r="B32" s="47" t="n">
-        <v>0.96</v>
+          <t>Production Value per Hour</t>
+        </is>
+      </c>
+      <c r="B32" s="48" t="n">
+        <v>4500</v>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
+          <t>USD/hr</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Finance — fully-loaded production cost model</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Downtime Cost = Value/hr × MTTR hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SUPPLIER COST MODEL INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Source / Basis</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Date Validated</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Supplier Margin – Low</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Engineering process spec</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Benchmarking; competitive-bid suppliers</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>Used in capacity model to calculate effective throughput</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>Production Value per Hour</t>
-        </is>
-      </c>
-      <c r="B33" s="48" t="n">
-        <v>4500</v>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>USD/hr</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Finance — fully-loaded production cost model</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>Downtime Cost = Value/hr × MTTR hrs</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>SUPPLIER COST MODEL INPUTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Source / Basis</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Date Validated</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Lower bound; applied to multi-source components</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Supplier Margin – Low</t>
+          <t>Supplier Margin – High</t>
         </is>
       </c>
       <c r="B37" s="47" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
@@ -35694,7 +35692,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Benchmarking; competitive-bid suppliers</t>
+          <t>Benchmarking; sole-source suppliers</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -35704,18 +35702,18 @@
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>Lower bound; applied to multi-source components</t>
+          <t>Upper bound; applied to single-source components</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Supplier Margin – High</t>
+          <t>Material Scrap Factor – Low</t>
         </is>
       </c>
       <c r="B38" s="47" t="n">
-        <v>0.25</v>
+        <v>0.05</v>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
@@ -35724,7 +35722,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Benchmarking; sole-source suppliers</t>
+          <t>Engineering; precision machined parts</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -35734,18 +35732,18 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>Upper bound; applied to single-source components</t>
+          <t>5% scrap on raw material purchases</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Material Scrap Factor – Low</t>
+          <t>Material Scrap Factor – High</t>
         </is>
       </c>
       <c r="B39" s="47" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
@@ -35754,7 +35752,7 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Engineering; precision machined parts</t>
+          <t>Engineering; cast / welded assemblies</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -35764,27 +35762,27 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>5% scrap on raw material purchases</t>
+          <t>8% scrap on complex fabrications</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Material Scrap Factor – High</t>
-        </is>
-      </c>
-      <c r="B40" s="47" t="n">
-        <v>0.08</v>
+          <t>Material Price – Steel (304 SS)</t>
+        </is>
+      </c>
+      <c r="B40" s="52" t="n">
+        <v>3.8</v>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>USD/kg</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Engineering; cast / welded assemblies</t>
+          <t>Metal bulletin Q1-2025</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
@@ -35794,18 +35792,18 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>8% scrap on complex fabrications</t>
+          <t>Used in vacuum chamber and furnace body cost estimates</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Material Price – Steel (304 SS)</t>
+          <t>Material Price – Aluminum</t>
         </is>
       </c>
       <c r="B41" s="52" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
@@ -35824,18 +35822,18 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>Used in vacuum chamber and furnace body cost estimates</t>
+          <t>Used in robotics frame and structural components</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Material Price – Aluminum</t>
+          <t>Material Price – Copper</t>
         </is>
       </c>
       <c r="B42" s="52" t="n">
-        <v>4.2</v>
+        <v>9.5</v>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
@@ -35844,7 +35842,7 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Metal bulletin Q1-2025</t>
+          <t>COMEX spot Q1-2025</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
@@ -35854,87 +35852,87 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>Used in robotics frame and structural components</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>Material Price – Copper</t>
-        </is>
-      </c>
-      <c r="B43" s="52" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>USD/kg</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>COMEX spot Q1-2025</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
+          <t>Used in transformer winding and electrical bus cost estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DEPLOYMENT TIMELINE ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Source / Basis</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Date Validated</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Supplier Manufacturing Duration</t>
+        </is>
+      </c>
+      <c r="B46" s="43" t="n">
+        <v>20</v>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Program schedule baseline Rev 1.0</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>Used in transformer winding and electrical bus cost estimates</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>DEPLOYMENT TIMELINE ASSUMPTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Source / Basis</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Date Validated</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Range: 16–24 wks depending on equipment complexity</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Supplier Manufacturing Duration</t>
+          <t>Factory Acceptance Testing (FAT)</t>
         </is>
       </c>
       <c r="B47" s="43" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
@@ -35943,7 +35941,7 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Program schedule baseline Rev 1.0</t>
+          <t>Standard FAT protocol – all equipment</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -35953,18 +35951,18 @@
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>Range: 16–24 wks depending on equipment complexity</t>
+          <t>2 weeks minimum; may extend for complex systems</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Factory Acceptance Testing (FAT)</t>
+          <t>International Shipping Duration</t>
         </is>
       </c>
       <c r="B48" s="43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
@@ -35973,7 +35971,7 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Standard FAT protocol – all equipment</t>
+          <t>Freight forwarder estimate; ocean freight</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -35983,18 +35981,18 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>2 weeks minimum; may extend for complex systems</t>
+          <t>Air freight contingency +50% cost; used for risk scenario</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>International Shipping Duration</t>
+          <t>On-Site Installation</t>
         </is>
       </c>
       <c r="B49" s="43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
@@ -36003,7 +36001,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Freight forwarder estimate; ocean freight</t>
+          <t>Facilities project plan Rev A</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -36013,18 +36011,18 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>Air freight contingency +50% cost; used for risk scenario</t>
+          <t>Per equipment platform; parallel installation possible</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>On-Site Installation</t>
+          <t>Utility Hookup</t>
         </is>
       </c>
       <c r="B50" s="43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
@@ -36033,7 +36031,7 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Facilities project plan Rev A</t>
+          <t>Facilities electrical + mechanical schedule</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
@@ -36043,18 +36041,18 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>Per equipment platform; parallel installation possible</t>
+          <t>Includes inspection and commissioning sign-off</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Utility Hookup</t>
+          <t>Process Qualification (PQ)</t>
         </is>
       </c>
       <c r="B51" s="43" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
@@ -36063,7 +36061,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Facilities electrical + mechanical schedule</t>
+          <t>Process engineering qualification plan</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -36073,91 +36071,91 @@
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>Includes inspection and commissioning sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>Process Qualification (PQ)</t>
-        </is>
-      </c>
-      <c r="B52" s="43" t="n">
-        <v>5</v>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>Weeks</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>Process engineering qualification plan</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
+          <t>Range: 4–6 wks; 5 wks used as baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>FX SENSITIVITY ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Source / Basis</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Date Validated</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>USD/EUR Exchange Rate (Baseline)</t>
+        </is>
+      </c>
+      <c r="B55" s="52" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>USD per EUR</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Bloomberg rates Q1-2025 average</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>Range: 4–6 wks; 5 wks used as baseline</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>FX SENSITIVITY ASSUMPTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Source / Basis</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>Date Validated</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>Baseline conversion rate for EUR-denominated equipment</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>USD/EUR Exchange Rate (Baseline)</t>
-        </is>
-      </c>
-      <c r="B56" s="52" t="n">
-        <v>1.09</v>
+          <t>USD/JPY Exchange Rate (Baseline)</t>
+        </is>
+      </c>
+      <c r="B56" s="43" t="n">
+        <v>149.5</v>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>USD per EUR</t>
+          <t>JPY per USD</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
@@ -36172,27 +36170,27 @@
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>Baseline conversion rate for EUR-denominated equipment</t>
+          <t>Baseline conversion rate for JPY-denominated equipment</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>USD/JPY Exchange Rate (Baseline)</t>
-        </is>
-      </c>
-      <c r="B57" s="43" t="n">
-        <v>149.5</v>
+          <t>EUR Sensitivity – Adverse</t>
+        </is>
+      </c>
+      <c r="B57" s="52" t="n">
+        <v>1.15</v>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>JPY per USD</t>
+          <t>USD per EUR</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Bloomberg rates Q1-2025 average</t>
+          <t>FX stress scenario +6%</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -36202,18 +36200,18 @@
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>Baseline conversion rate for JPY-denominated equipment</t>
+          <t>1% move in EUR/USD = ~$85K portfolio cost impact</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>EUR Sensitivity – Adverse</t>
+          <t>EUR Sensitivity – Favorable</t>
         </is>
       </c>
       <c r="B58" s="52" t="n">
-        <v>1.15</v>
+        <v>1.03</v>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
@@ -36222,7 +36220,7 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>FX stress scenario +6%</t>
+          <t>FX stress scenario -6%</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
@@ -36232,27 +36230,27 @@
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>1% move in EUR/USD = ~$85K portfolio cost impact</t>
+          <t>Favorable scenario used in S13 Scenario Analysis</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>EUR Sensitivity – Favorable</t>
-        </is>
-      </c>
-      <c r="B59" s="52" t="n">
-        <v>1.03</v>
+          <t>JPY Sensitivity – Adverse</t>
+        </is>
+      </c>
+      <c r="B59" s="43" t="n">
+        <v>142</v>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>USD per EUR</t>
+          <t>JPY per USD</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>FX stress scenario -6%</t>
+          <t>FX stress scenario (JPY strengthens)</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
@@ -36262,18 +36260,18 @@
       </c>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>Favorable scenario used in S13 Scenario Analysis</t>
+          <t>Stronger JPY = higher USD cost for JPY equipment</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>JPY Sensitivity – Adverse</t>
+          <t>JPY Sensitivity – Favorable</t>
         </is>
       </c>
       <c r="B60" s="43" t="n">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
@@ -36282,7 +36280,7 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>FX stress scenario (JPY strengthens)</t>
+          <t>FX stress scenario (JPY weakens)</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
@@ -36292,108 +36290,115 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Stronger JPY = higher USD cost for JPY equipment</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t>JPY Sensitivity – Favorable</t>
-        </is>
-      </c>
-      <c r="B61" s="43" t="n">
-        <v>157</v>
-      </c>
-      <c r="C61" s="6" t="inlineStr">
-        <is>
-          <t>JPY per USD</t>
-        </is>
-      </c>
-      <c r="D61" s="6" t="inlineStr">
-        <is>
-          <t>FX stress scenario (JPY weakens)</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="F61" s="8" t="inlineStr">
-        <is>
           <t>Weaker JPY = lower USD cost for JPY equipment</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>VERSION CONTROL LOG — Model Revision History &amp; Change Tracking</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="5" t="inlineStr">
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B64" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Owner / Author</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Change Description</t>
         </is>
       </c>
-      <c r="E64" s="5" t="inlineStr">
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>Impact on Model</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr">
+      <c r="F63" s="5" t="inlineStr">
         <is>
           <t>Approval Status</t>
         </is>
       </c>
-      <c r="G64" s="5" t="inlineStr">
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>Notes / Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>V1.0</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>2025-02-10</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Sourabh Tarodekar (TPM)</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Initial workbook created. Equipment portfolio dataset populated with 15 platforms from supplier quotes.</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Baseline established. All formulas reference V1.0 assumptions.</t>
+        </is>
+      </c>
+      <c r="F64" s="40" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="inlineStr">
+        <is>
+          <t>Baseline model — AR-2025-0082 submission basis</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>V1.0</t>
+          <t>V1.1</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>2025-02-10</t>
+          <t>2025-02-14</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Sourabh Tarodekar (TPM)</t>
+          <t>S. Kim (Supply Chain)</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>Initial workbook created. Equipment portfolio dataset populated with 15 platforms from supplier quotes.</t>
+          <t>Updated Pfeiffer vacuum pump (EQ-002) lead time from 16 to 26 weeks based on supplier confirmation.</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Baseline established. All formulas reference V1.0 assumptions.</t>
+          <t>Deployment timeline extended. EQ-002 now on critical path. Risk flag updated to CRITICAL.</t>
         </is>
       </c>
       <c r="F65" s="40" t="inlineStr">
@@ -36403,34 +36408,34 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Baseline model — AR-2025-0082 submission basis</t>
+          <t>Supplier email confirmation 2025-02-13 on file</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>V1.1</t>
+          <t>V1.2</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>2025-02-18</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>S. Kim (Supply Chain)</t>
+          <t>R. Patel (Finance)</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Updated Pfeiffer vacuum pump (EQ-002) lead time from 16 to 26 weeks based on supplier confirmation.</t>
+          <t>Discount rate updated from 7.5% to 8.0% per Q1-2025 corporate WACC guidance.</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Deployment timeline extended. EQ-002 now on critical path. Risk flag updated to CRITICAL.</t>
+          <t>NPV reduced by ~$420K. TCO model and scenario analysis recalculated.</t>
         </is>
       </c>
       <c r="F66" s="40" t="inlineStr">
@@ -36440,34 +36445,34 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Supplier email confirmation 2025-02-13 on file</t>
+          <t>Finance guidance memo FIN-2025-007</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>V1.2</t>
+          <t>V1.3</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>2025-02-18</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>R. Patel (Finance)</t>
+          <t>T. Okonkwo (Facilities)</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>Discount rate updated from 7.5% to 8.0% per Q1-2025 corporate WACC guidance.</t>
+          <t>Added EQ-004 crane hire and floor reinforcement to installation cost — +$62K.</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>NPV reduced by ~$420K. TCO model and scenario analysis recalculated.</t>
+          <t>Total installation cost increased. CR-001 raised. Change tracker updated.</t>
         </is>
       </c>
       <c r="F67" s="40" t="inlineStr">
@@ -36477,34 +36482,34 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>Finance guidance memo FIN-2025-007</t>
+          <t>CR-001 approved by PM 2025-02-24</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>V1.3</t>
+          <t>V1.4</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>2025-03-05</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>T. Okonkwo (Facilities)</t>
+          <t>M. Chen (Process Eng.)</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Added EQ-004 crane hire and floor reinforcement to installation cost — +$62K.</t>
+          <t>Equipment uptime revised from 90% to 92% following process engineering specification review.</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>Total installation cost increased. CR-001 raised. Change tracker updated.</t>
+          <t>Annual capacity increased. Utilization % reduced. Capacity model updated.</t>
         </is>
       </c>
       <c r="F68" s="40" t="inlineStr">
@@ -36514,34 +36519,34 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>CR-001 approved by PM 2025-02-24</t>
+          <t>Process spec document PE-2025-014 Rev A</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>V1.4</t>
+          <t>V1.5</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>2025-03-10</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>M. Chen (Process Eng.)</t>
+          <t>R. Patel (Finance)</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Equipment uptime revised from 90% to 92% following process engineering specification review.</t>
+          <t>FX sensitivity assumptions added. EUR/JPY baseline and stress scenarios populated.</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>Annual capacity increased. Utilization % reduced. Capacity model updated.</t>
+          <t>FX exposure model now active. EUR/USD baseline 1.09, JPY/USD baseline 149.5.</t>
         </is>
       </c>
       <c r="F69" s="40" t="inlineStr">
@@ -36551,34 +36556,34 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Process spec document PE-2025-014 Rev A</t>
+          <t>Bloomberg rates Q1-2025 average</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>V1.5</t>
+          <t>V1.6</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2025-03-17</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>R. Patel (Finance)</t>
+          <t>S. Kim (Supply Chain)</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>FX sensitivity assumptions added. EUR/JPY baseline and stress scenarios populated.</t>
+          <t>Supplier risk scores recalculated after Daifuku confirmed 30-week manufacturing lead time for EQ-006.</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>FX exposure model now active. EUR/USD baseline 1.09, JPY/USD baseline 149.5.</t>
+          <t>EQ-006 risk tier escalated to CRITICAL. Supply chain risk index increased.</t>
         </is>
       </c>
       <c r="F70" s="40" t="inlineStr">
@@ -36588,34 +36593,34 @@
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Bloomberg rates Q1-2025 average</t>
+          <t>Daifuku PO confirmation email</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>V1.6</t>
+          <t>V1.7</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>2025-03-17</t>
+          <t>2025-03-19</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>S. Kim (Supply Chain)</t>
+          <t>Sourabh Tarodekar (TPM)</t>
         </is>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Supplier risk scores recalculated after Daifuku confirmed 30-week manufacturing lead time for EQ-006.</t>
+          <t>AR Summary populated and submitted to VP Engineering + CFO. Budget: $40.04M (Scenario B benchmark).</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>EQ-006 risk tier escalated to CRITICAL. Supply chain risk index increased.</t>
+          <t>Formal program approval process initiated. Model frozen for AR submission.</t>
         </is>
       </c>
       <c r="F71" s="40" t="inlineStr">
@@ -36625,34 +36630,34 @@
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>Daifuku PO confirmation email</t>
+          <t>AR-2025-0082 submitted to Finance</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>V1.7</t>
+          <t>V1.8</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>2025-03-19</t>
+          <t>2025-04-05</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Sourabh Tarodekar (TPM)</t>
+          <t>R. Patel (Finance)</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>AR Summary populated and submitted to VP Engineering + CFO. Budget: $40.04M (Scenario B benchmark).</t>
+          <t>AR approved. POs placed for long-lead items. Spend tracking model activated.</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>Formal program approval process initiated. Model frozen for AR submission.</t>
+          <t>Program execution phase begins. Cash flow schedule now active.</t>
         </is>
       </c>
       <c r="F72" s="40" t="inlineStr">
@@ -36662,116 +36667,79 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>AR-2025-0082 submitted to Finance</t>
+          <t>CFO approval email 2025-04-05</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>V1.8</t>
+          <t>V1.9</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>2025-04-05</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>R. Patel (Finance)</t>
+          <t>P. Singh (IT/OT)</t>
         </is>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>AR approved. POs placed for long-lead items. Spend tracking model activated.</t>
+          <t>IT/OT DMZ infrastructure cost ($45K) added to scope. CR-009 raised.</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>Program execution phase begins. Cash flow schedule now active.</t>
-        </is>
-      </c>
-      <c r="F73" s="40" t="inlineStr">
-        <is>
-          <t>APPROVED</t>
+          <t>Contingency draw of $45K. Change tracker updated. Contingency at 5.8%.</t>
+        </is>
+      </c>
+      <c r="F73" s="46" t="inlineStr">
+        <is>
+          <t>UNDER REVIEW</t>
         </is>
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>CFO approval email 2025-04-05</t>
+          <t>CR-009 pending PM approval</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>V1.9</t>
+          <t>V2.0</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>2025-05-19</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>P. Singh (IT/OT)</t>
+          <t>Sourabh Tarodekar (TPM)</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>IT/OT DMZ infrastructure cost ($45K) added to scope. CR-009 raised.</t>
+          <t>Version 2.0 release: Cash flow schedule, FX exposure model, and ROI tracker sheets added.</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>Contingency draw of $45K. Change tracker updated. Contingency at 5.8%.</t>
-        </is>
-      </c>
-      <c r="F74" s="46" t="inlineStr">
-        <is>
-          <t>UNDER REVIEW</t>
+          <t>Workbook extended with 4 new analytical sheets. Full model refresh completed.</t>
+        </is>
+      </c>
+      <c r="F74" s="40" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
         </is>
       </c>
       <c r="G74" s="8" t="inlineStr">
-        <is>
-          <t>CR-009 pending PM approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>V2.0</t>
-        </is>
-      </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>2025-05-19</t>
-        </is>
-      </c>
-      <c r="C75" s="6" t="inlineStr">
-        <is>
-          <t>Sourabh Tarodekar (TPM)</t>
-        </is>
-      </c>
-      <c r="D75" s="8" t="inlineStr">
-        <is>
-          <t>Version 2.0 release: Cash flow schedule, FX exposure model, and ROI tracker sheets added.</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>Workbook extended with 4 new analytical sheets. Full model refresh completed.</t>
-        </is>
-      </c>
-      <c r="F75" s="40" t="inlineStr">
-        <is>
-          <t>APPROVED</t>
-        </is>
-      </c>
-      <c r="G75" s="8" t="inlineStr">
         <is>
           <t>Issued to Finance and Engineering Leadership</t>
         </is>
@@ -36780,16 +36748,16 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A62:G62"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A53:F53"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -40813,7 +40781,7 @@
         <v/>
       </c>
       <c r="L5" s="41">
-        <f>(J5+K5)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J5+K5)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M5" s="31">
@@ -40851,7 +40819,7 @@
         <v>95</v>
       </c>
       <c r="G6" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H6" s="31">
@@ -40870,7 +40838,7 @@
         <v/>
       </c>
       <c r="L6" s="41">
-        <f>(J6+K6)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J6+K6)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M6" s="31">
@@ -40926,7 +40894,7 @@
         <v/>
       </c>
       <c r="L7" s="41">
-        <f>(J7+K7)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J7+K7)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M7" s="31">
@@ -40982,7 +40950,7 @@
         <v/>
       </c>
       <c r="L8" s="41">
-        <f>(J8+K8)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J8+K8)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M8" s="31">
@@ -41020,7 +40988,7 @@
         <v>32</v>
       </c>
       <c r="G9" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H9" s="31">
@@ -41039,7 +41007,7 @@
         <v/>
       </c>
       <c r="L9" s="41">
-        <f>(J9+K9)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J9+K9)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M9" s="31">
@@ -41077,7 +41045,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$24</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
         <v/>
       </c>
       <c r="H10" s="31">
@@ -41096,7 +41064,7 @@
         <v/>
       </c>
       <c r="L10" s="41">
-        <f>(J10+K10)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J10+K10)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M10" s="31">
@@ -41152,7 +41120,7 @@
         <v/>
       </c>
       <c r="L11" s="41">
-        <f>(J11+K11)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J11+K11)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M11" s="31">
@@ -41190,7 +41158,7 @@
         <v>180</v>
       </c>
       <c r="G12" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H12" s="31">
@@ -41209,7 +41177,7 @@
         <v/>
       </c>
       <c r="L12" s="41">
-        <f>(J12+K12)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J12+K12)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M12" s="31">
@@ -41265,7 +41233,7 @@
         <v/>
       </c>
       <c r="L13" s="41">
-        <f>(J13+K13)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J13+K13)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M13" s="31">
@@ -41321,7 +41289,7 @@
         <v/>
       </c>
       <c r="L14" s="41">
-        <f>(J14+K14)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J14+K14)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M14" s="31">
@@ -41359,7 +41327,7 @@
         <v>65</v>
       </c>
       <c r="G15" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H15" s="31">
@@ -41378,7 +41346,7 @@
         <v/>
       </c>
       <c r="L15" s="41">
-        <f>(J15+K15)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J15+K15)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M15" s="31">
@@ -41416,7 +41384,7 @@
         <v>20</v>
       </c>
       <c r="G16" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$24</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
         <v/>
       </c>
       <c r="H16" s="31">
@@ -41435,7 +41403,7 @@
         <v/>
       </c>
       <c r="L16" s="41">
-        <f>(J16+K16)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J16+K16)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M16" s="31">
@@ -41491,7 +41459,7 @@
         <v/>
       </c>
       <c r="L17" s="41">
-        <f>(J17+K17)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J17+K17)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M17" s="31">
@@ -41529,7 +41497,7 @@
         <v>40</v>
       </c>
       <c r="G18" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H18" s="31">
@@ -41548,7 +41516,7 @@
         <v/>
       </c>
       <c r="L18" s="41">
-        <f>(J18+K18)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J18+K18)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M18" s="31">
@@ -41604,7 +41572,7 @@
         <v/>
       </c>
       <c r="L19" s="41">
-        <f>(J19+K19)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J19+K19)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M19" s="31">
@@ -41660,7 +41628,7 @@
         <v/>
       </c>
       <c r="L20" s="41">
-        <f>(J20+K20)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J20+K20)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M20" s="31">
@@ -41698,7 +41666,7 @@
         <v>35</v>
       </c>
       <c r="G21" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$24</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
         <v/>
       </c>
       <c r="H21" s="31">
@@ -41717,7 +41685,7 @@
         <v/>
       </c>
       <c r="L21" s="41">
-        <f>(J21+K21)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J21+K21)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M21" s="31">
@@ -41755,7 +41723,7 @@
         <v>10</v>
       </c>
       <c r="G22" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$24</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
         <v/>
       </c>
       <c r="H22" s="31">
@@ -41774,7 +41742,7 @@
         <v/>
       </c>
       <c r="L22" s="41">
-        <f>(J22+K22)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J22+K22)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M22" s="31">
@@ -41830,7 +41798,7 @@
         <v/>
       </c>
       <c r="L23" s="41">
-        <f>(J23+K23)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J23+K23)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M23" s="31">
@@ -41868,7 +41836,7 @@
         <v>55</v>
       </c>
       <c r="G24" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H24" s="31">
@@ -41887,7 +41855,7 @@
         <v/>
       </c>
       <c r="L24" s="41">
-        <f>(J24+K24)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J24+K24)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M24" s="31">
@@ -41943,7 +41911,7 @@
         <v/>
       </c>
       <c r="L25" s="41">
-        <f>(J25+K25)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J25+K25)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M25" s="31">
@@ -41999,7 +41967,7 @@
         <v/>
       </c>
       <c r="L26" s="41">
-        <f>(J26+K26)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J26+K26)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M26" s="31">
@@ -42037,7 +42005,7 @@
         <v>28</v>
       </c>
       <c r="G27" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H27" s="31">
@@ -42056,7 +42024,7 @@
         <v/>
       </c>
       <c r="L27" s="41">
-        <f>(J27+K27)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J27+K27)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M27" s="31">
@@ -42094,7 +42062,7 @@
         <v>8</v>
       </c>
       <c r="G28" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$24</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
         <v/>
       </c>
       <c r="H28" s="31">
@@ -42113,7 +42081,7 @@
         <v/>
       </c>
       <c r="L28" s="41">
-        <f>(J28+K28)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J28+K28)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M28" s="31">
@@ -42169,7 +42137,7 @@
         <v/>
       </c>
       <c r="L29" s="41">
-        <f>(J29+K29)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J29+K29)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M29" s="31">
@@ -42207,7 +42175,7 @@
         <v>45</v>
       </c>
       <c r="G30" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$22</f>
         <v/>
       </c>
       <c r="H30" s="31">
@@ -42226,7 +42194,7 @@
         <v/>
       </c>
       <c r="L30" s="41">
-        <f>(J30+K30)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J30+K30)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M30" s="31">
@@ -42264,7 +42232,7 @@
         <v>80</v>
       </c>
       <c r="G31" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$24</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
         <v/>
       </c>
       <c r="H31" s="31">
@@ -42283,7 +42251,7 @@
         <v/>
       </c>
       <c r="L31" s="41">
-        <f>(J31+K31)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J31+K31)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M31" s="31">
@@ -42321,7 +42289,7 @@
         <v>16</v>
       </c>
       <c r="G32" s="60">
-        <f>'S01_Disclaimer_Assumptions'!$B$24</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$23</f>
         <v/>
       </c>
       <c r="H32" s="31">
@@ -42340,7 +42308,7 @@
         <v/>
       </c>
       <c r="L32" s="41">
-        <f>(J32+K32)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(J32+K32)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="M32" s="31">
@@ -42444,7 +42412,7 @@
         <v/>
       </c>
       <c r="G36" s="31">
-        <f>(E36+F36)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(E36+F36)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="H36" s="31">
@@ -42490,7 +42458,7 @@
         <v/>
       </c>
       <c r="G37" s="31">
-        <f>(E37+F37)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(E37+F37)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="H37" s="31">
@@ -42536,7 +42504,7 @@
         <v/>
       </c>
       <c r="G38" s="31">
-        <f>(E38+F38)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(E38+F38)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="H38" s="31">
@@ -42582,7 +42550,7 @@
         <v/>
       </c>
       <c r="G39" s="31">
-        <f>(E39+F39)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(E39+F39)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="H39" s="31">
@@ -42628,7 +42596,7 @@
         <v/>
       </c>
       <c r="G40" s="31">
-        <f>(E40+F40)*'S01_Disclaimer_Assumptions'!$B$38</f>
+        <f>(E40+F40)*'S01_Disclaimer_Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="H40" s="31">
@@ -42789,7 +42757,7 @@
         </is>
       </c>
       <c r="B8" s="64">
-        <f>'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
     </row>
@@ -42800,7 +42768,7 @@
         </is>
       </c>
       <c r="B9" s="62">
-        <f>'S01_Disclaimer_Assumptions'!$B$19</f>
+        <f>'S01_Disclaimer_Assumptions'!$B$18</f>
         <v/>
       </c>
     </row>
@@ -43370,39 +43338,39 @@
         <v/>
       </c>
       <c r="C34" s="31">
-        <f>B34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>B34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="D34" s="31">
-        <f>C34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>C34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="E34" s="31">
-        <f>D34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>D34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="F34" s="31">
-        <f>E34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>E34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="G34" s="31">
-        <f>F34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>F34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="H34" s="31">
-        <f>G34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>G34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="I34" s="31">
-        <f>H34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>H34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="J34" s="31">
-        <f>I34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>I34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="K34" s="31">
-        <f>J34*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>J34*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="L34" s="31">
@@ -43425,39 +43393,39 @@
         <v/>
       </c>
       <c r="C35" s="31">
-        <f>B35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>B35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="D35" s="31">
-        <f>C35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>C35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="E35" s="31">
-        <f>D35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>D35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="F35" s="31">
-        <f>E35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>E35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="G35" s="31">
-        <f>F35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>F35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="H35" s="31">
-        <f>G35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>G35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="I35" s="31">
-        <f>H35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>H35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="J35" s="31">
-        <f>I35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>I35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="K35" s="31">
-        <f>J35*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>J35*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="L35" s="31">
@@ -43487,39 +43455,39 @@
         <v/>
       </c>
       <c r="C37" s="31">
-        <f>B37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>B37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="D37" s="31">
-        <f>C37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>C37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="E37" s="31">
-        <f>D37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>D37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="F37" s="31">
-        <f>E37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>E37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="G37" s="31">
-        <f>F37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>F37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="H37" s="31">
-        <f>G37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>G37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="I37" s="31">
-        <f>H37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>H37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="J37" s="31">
-        <f>I37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>I37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="K37" s="31">
-        <f>J37*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>J37*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="L37" s="31">
@@ -43542,39 +43510,39 @@
         <v/>
       </c>
       <c r="C38" s="31">
-        <f>B38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>B38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="D38" s="31">
-        <f>C38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>C38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="E38" s="31">
-        <f>D38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>D38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="F38" s="31">
-        <f>E38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>E38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="G38" s="31">
-        <f>F38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>F38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="H38" s="31">
-        <f>G38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>G38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="I38" s="31">
-        <f>H38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>H38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="J38" s="31">
-        <f>I38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>I38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="K38" s="31">
-        <f>J38*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>J38*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="L38" s="31">
@@ -43604,39 +43572,39 @@
         <v/>
       </c>
       <c r="C40" s="31">
-        <f>B40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>B40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="D40" s="31">
-        <f>C40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>C40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="E40" s="31">
-        <f>D40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>D40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="F40" s="31">
-        <f>E40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>E40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="G40" s="31">
-        <f>F40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>F40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="H40" s="31">
-        <f>G40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>G40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="I40" s="31">
-        <f>H40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>H40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="J40" s="31">
-        <f>I40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>I40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="K40" s="31">
-        <f>J40*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>J40*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="L40" s="31">
@@ -43659,39 +43627,39 @@
         <v/>
       </c>
       <c r="C41" s="31">
-        <f>B41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>B41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="D41" s="31">
-        <f>C41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>C41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="E41" s="31">
-        <f>D41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>D41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="F41" s="31">
-        <f>E41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>E41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="G41" s="31">
-        <f>F41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>F41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="H41" s="31">
-        <f>G41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>G41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="I41" s="31">
-        <f>H41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>H41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="J41" s="31">
-        <f>I41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>I41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="K41" s="31">
-        <f>J41*(1+'S01_Disclaimer_Assumptions'!$B$19)</f>
+        <f>J41*(1+'S01_Disclaimer_Assumptions'!$B$18)</f>
         <v/>
       </c>
       <c r="L41" s="31">
@@ -43717,43 +43685,43 @@
         </is>
       </c>
       <c r="B43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="C43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="D43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="E43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="F43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="G43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="H43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="I43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="J43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="K43" s="31">
-        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/4200)*6*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="L43" s="31">
@@ -43772,43 +43740,43 @@
         </is>
       </c>
       <c r="B44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="C44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="D44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="E44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="F44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="G44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="H44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="I44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="J44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="K44" s="31">
-        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$33</f>
+        <f>(8320/2800)*10*'S01_Disclaimer_Assumptions'!$B$32</f>
         <v/>
       </c>
       <c r="L44" s="31">

</xml_diff>